<commit_message>
use boot package for bias-adjusted bootstrap, use permutation test for p-values
</commit_message>
<xml_diff>
--- a/0-Config/0-Files/var_name_mapping.xlsx
+++ b/0-Config/0-Files/var_name_mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maggiewang/Documents/stanford/repos/woebot/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maggiewang/Documents/stanford/repos/woebot/0-Config/0-Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09E2E5D2-7508-9147-BA13-F4F2B82D93F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9029AD07-5C00-6847-B036-B0C0CD4CACE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="baseline" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="703">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="704">
   <si>
     <t>var_name</t>
   </si>
@@ -2133,6 +2133,9 @@
   </si>
   <si>
     <t>tq34</t>
+  </si>
+  <si>
+    <t>emailaddress</t>
   </si>
 </sst>
 </file>
@@ -2691,9 +2694,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2731,7 +2734,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2837,7 +2840,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2979,7 +2982,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -30387,7 +30390,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C69C1F0A-5582-4842-9906-AF7DC99E3E7B}">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.83203125" bestFit="1" customWidth="1"/>
@@ -30483,6 +30486,11 @@
         <v>572</v>
       </c>
     </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>703</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>